<commit_message>
setup for test5 env.
</commit_message>
<xml_diff>
--- a/EU/DataSheet.xlsx
+++ b/EU/DataSheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://libertymutual-my.sharepoint.com/personal/mohammad_talib_libertymutual_com/Documents/Desktop/regression-pack/EU/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="19" documentId="6_{458F8D31-B834-481D-A478-E53F0DAC6831}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{63002CCE-A111-4EEC-AE74-8CAD6856AEF5}"/>
+  <xr:revisionPtr revIDLastSave="23" documentId="6_{458F8D31-B834-481D-A478-E53F0DAC6831}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A10ACB93-4505-40A7-ABDD-0FAF627E2B2C}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="2" xr2:uid="{A2EF6AEE-92DE-49D8-BB60-1A120F6353A4}"/>
   </bookViews>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2177" uniqueCount="674">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2177" uniqueCount="675">
   <si>
     <t>First Named Insured</t>
   </si>
@@ -2076,6 +2076,9 @@
   </si>
   <si>
     <t>15/09/2025</t>
+  </si>
+  <si>
+    <t>https://n9971008:wm$qY@08@test5-underwritingplatform.grsazr.lmig.com</t>
   </si>
 </sst>
 </file>
@@ -9569,7 +9572,7 @@
     <col min="47" max="47" width="23.42578125" style="11" bestFit="1" customWidth="1"/>
     <col min="48" max="48" width="18.85546875" style="11" bestFit="1" customWidth="1"/>
     <col min="49" max="49" width="11.5703125" style="11" bestFit="1" customWidth="1"/>
-    <col min="50" max="50" width="9.5703125" style="11" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="10.5703125" style="11" bestFit="1" customWidth="1"/>
     <col min="51" max="16384" width="9.140625" style="11"/>
   </cols>
   <sheetData>
@@ -9792,7 +9795,7 @@
     </row>
     <row r="3" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A3" s="18" t="s">
-        <v>592</v>
+        <v>674</v>
       </c>
       <c r="B3" t="s">
         <v>584</v>
@@ -9939,7 +9942,7 @@
         <v>613</v>
       </c>
       <c r="AX3" s="46">
-        <v>46263</v>
+        <v>46337</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
setup for hfstage env.
</commit_message>
<xml_diff>
--- a/EU/DataSheet.xlsx
+++ b/EU/DataSheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://libertymutual-my.sharepoint.com/personal/mohammad_talib_libertymutual_com/Documents/Desktop/regression-pack/EU/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="24" documentId="6_{458F8D31-B834-481D-A478-E53F0DAC6831}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{921D51ED-AE50-415C-9370-6C6F6E2AFFC8}"/>
+  <xr:revisionPtr revIDLastSave="25" documentId="6_{458F8D31-B834-481D-A478-E53F0DAC6831}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{154D4CA7-8F57-4074-8CBB-1713732E047C}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="2" xr2:uid="{A2EF6AEE-92DE-49D8-BB60-1A120F6353A4}"/>
   </bookViews>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2177" uniqueCount="674">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2177" uniqueCount="675">
   <si>
     <t>First Named Insured</t>
   </si>
@@ -2076,6 +2076,9 @@
   </si>
   <si>
     <t>15/09/2025</t>
+  </si>
+  <si>
+    <t>https://n9971008:wm$qY@08@hfstage-underwritingplatform.grsazr.lmig.com</t>
   </si>
 </sst>
 </file>
@@ -9792,7 +9795,7 @@
     </row>
     <row r="3" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A3" s="18" t="s">
-        <v>592</v>
+        <v>674</v>
       </c>
       <c r="B3" t="s">
         <v>584</v>

</xml_diff>

<commit_message>
setup for test env for regression.
</commit_message>
<xml_diff>
--- a/EU/DataSheet.xlsx
+++ b/EU/DataSheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://libertymutual-my.sharepoint.com/personal/mohammad_talib_libertymutual_com/Documents/Desktop/regression-pack/EU/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="24" documentId="6_{458F8D31-B834-481D-A478-E53F0DAC6831}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{921D51ED-AE50-415C-9370-6C6F6E2AFFC8}"/>
+  <xr:revisionPtr revIDLastSave="27" documentId="6_{458F8D31-B834-481D-A478-E53F0DAC6831}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3C2D2B43-331B-4678-B753-51438B7A2F4B}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="2" xr2:uid="{A2EF6AEE-92DE-49D8-BB60-1A120F6353A4}"/>
   </bookViews>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2177" uniqueCount="674">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2177" uniqueCount="675">
   <si>
     <t>First Named Insured</t>
   </si>
@@ -2076,6 +2076,9 @@
   </si>
   <si>
     <t>15/09/2025</t>
+  </si>
+  <si>
+    <t>https://n9971008:wm$qY@08@test-underwritingplatform.grsazr.lmig.com</t>
   </si>
 </sst>
 </file>
@@ -9792,7 +9795,7 @@
     </row>
     <row r="3" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A3" s="18" t="s">
-        <v>592</v>
+        <v>674</v>
       </c>
       <c r="B3" t="s">
         <v>584</v>

</xml_diff>